<commit_message>
ADIB: workbook recalculates clean, document rebuilt on the class primary
</commit_message>
<xml_diff>
--- a/engine/adib_study/ADIB_Valuation_Model_09092026.xlsx
+++ b/engine/adib_study/ADIB_Valuation_Model_09092026.xlsx
@@ -1193,9 +1193,10 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4">
-        <f> Dividend</f>
-        <v/>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>equals the Dividend</t>
+        </is>
       </c>
       <c r="C7" s="6">
         <f>'Balance Sheet'!C13</f>
@@ -1246,9 +1247,10 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4">
-        <f> NET FLOW TO SHAREHOLDERS</f>
-        <v/>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>equals the NET FLOW TO SHAREHOLDERS</t>
+        </is>
       </c>
       <c r="C9" s="6">
         <f>'Balance Sheet'!C15</f>
@@ -3476,7 +3478,7 @@
         </is>
       </c>
       <c r="B24" s="6">
-        <f>(H21*(1+'Assumptions'!$B$28)/('Assumptions'!$B$31-'Assumptions'!$B$28))*H5</f>
+        <f>(('Income Statement'!I14-'Assumptions'!$B$31*'Balance Sheet'!G10)*(1+'Assumptions'!$B$28)/('Assumptions'!$B$31-'Assumptions'!$B$28))*H5</f>
         <v/>
       </c>
     </row>

</xml_diff>